<commit_message>
functionable - Login and out with session
</commit_message>
<xml_diff>
--- a/IMS_normalization.xlsx
+++ b/IMS_normalization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\IMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2232974A-E742-4371-A57F-DCD647817DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7658D334-ADBF-4CBD-B2A2-4166B7C5FF41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{2CDF4D7C-9BB1-444C-B0E6-E0178AB74584}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CDF4D7C-9BB1-444C-B0E6-E0178AB74584}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="107">
   <si>
     <t>ASSET</t>
   </si>
@@ -132,9 +132,6 @@
     <t>serial_number</t>
   </si>
   <si>
-    <t>text</t>
-  </si>
-  <si>
     <t>asset_ID PK</t>
   </si>
   <si>
@@ -153,9 +150,6 @@
     <t>brand_name</t>
   </si>
   <si>
-    <t>TEXT</t>
-  </si>
-  <si>
     <t>brand_ID PK</t>
   </si>
   <si>
@@ -295,13 +289,70 @@
   </si>
   <si>
     <t>user_ID FK</t>
+  </si>
+  <si>
+    <t>VARCHAR</t>
+  </si>
+  <si>
+    <t>Request</t>
+  </si>
+  <si>
+    <t>request_date</t>
+  </si>
+  <si>
+    <t>TIME</t>
+  </si>
+  <si>
+    <t>request_time</t>
+  </si>
+  <si>
+    <t>UOM</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>request_ID PK</t>
+  </si>
+  <si>
+    <t>unit_ID FK</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>request_note</t>
+  </si>
+  <si>
+    <t>KLD_ID</t>
+  </si>
+  <si>
+    <t>barcode_image_path_ID FK</t>
+  </si>
+  <si>
+    <t>Barcode</t>
+  </si>
+  <si>
+    <t>barcode_image_path_ID PK</t>
+  </si>
+  <si>
+    <t>barcode_image_path</t>
+  </si>
+  <si>
+    <t>asset_status</t>
+  </si>
+  <si>
+    <t>remember_token</t>
+  </si>
+  <si>
+    <t>token_expiry</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,6 +385,12 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -407,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -429,11 +486,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -442,15 +502,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -459,10 +525,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -779,14 +842,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DB240BC-D6BF-403C-8C3D-179145117FF2}">
-  <dimension ref="A2:J77"/>
+  <dimension ref="A2:J84"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" customWidth="1"/>
     <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.33203125" customWidth="1"/>
     <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
@@ -801,11 +864,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -910,25 +973,25 @@
       <c r="J6" s="4"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="D12" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E12" s="14"/>
-      <c r="H12" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="I12" s="10"/>
+      <c r="B12" s="18"/>
+      <c r="D12" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="19"/>
+      <c r="H12" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="I12" s="15"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
@@ -952,39 +1015,39 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>32</v>
@@ -992,71 +1055,71 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>35</v>
+        <v>88</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>33</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>35</v>
+        <v>88</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>34</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D19" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E19" s="15"/>
+      <c r="H19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D19" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E19" s="10"/>
-      <c r="H19" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="11"/>
       <c r="D20" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>30</v>
@@ -1067,42 +1130,42 @@
         <v>31</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B25" s="12"/>
+      <c r="B25" s="13"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
@@ -1114,40 +1177,40 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D30" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
+      <c r="D30" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="13"/>
-      <c r="D32" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E32" s="14"/>
-      <c r="H32" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="I32" s="10"/>
+      <c r="B32" s="18"/>
+      <c r="D32" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="19"/>
+      <c r="H32" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="I32" s="15"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
@@ -1171,39 +1234,39 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>32</v>
@@ -1211,94 +1274,94 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
-        <v>35</v>
+        <v>88</v>
       </c>
       <c r="B37" s="7" t="s">
         <v>33</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
-        <v>35</v>
+        <v>88</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D38" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E38" s="10"/>
+      <c r="D38" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E38" s="15"/>
       <c r="H38" s="2" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>30</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D40" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B41" s="12"/>
+      <c r="A41" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" s="13"/>
       <c r="D41" s="2" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
@@ -1311,24 +1374,24 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D43" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="E43" s="14"/>
-      <c r="H43" s="17"/>
-      <c r="I43" s="18"/>
+        <v>45</v>
+      </c>
+      <c r="D43" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E43" s="19"/>
+      <c r="H43" s="20"/>
+      <c r="I43" s="21"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>31</v>
@@ -1341,22 +1404,22 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D45" s="8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B46" s="16"/>
+      <c r="A46" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B46" s="11"/>
       <c r="D46" s="8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
@@ -1364,77 +1427,77 @@
         <v>31</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="7" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D50" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D54" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="E54" s="20"/>
-      <c r="F54" s="20"/>
+      <c r="D54" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="E54" s="17"/>
+      <c r="F54" s="17"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="13" t="s">
+      <c r="A56" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B56" s="13"/>
+      <c r="D56" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B56" s="13"/>
-      <c r="D56" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E56" s="14"/>
-      <c r="H56" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="I56" s="10"/>
+      <c r="E56" s="18"/>
+      <c r="H56" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="I56" s="15"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" s="6" t="s">
+      <c r="A57" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="B57" s="3" t="s">
         <v>30</v>
       </c>
       <c r="D57" s="6" t="s">
@@ -1451,323 +1514,451 @@
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B58" s="7" t="s">
+      <c r="A58" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E59" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D58" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E58" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="H58" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B59" s="7" t="s">
+      <c r="H59" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D60" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E60" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D59" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E59" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="H59" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="I59" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B60" s="7" t="s">
+      <c r="H60" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A61" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D60" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E60" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="I60" s="2" t="s">
+      <c r="B61" s="11"/>
+      <c r="D61" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A62" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I62" s="2" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B61" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E61" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I61" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A62" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B62" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D62" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E62" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="H62" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I62" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>64</v>
+        <v>41</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>62</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A64" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E64" s="9" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A65" s="11" t="s">
+      <c r="D65" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E65" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="H65" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="I65" s="15"/>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A66" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B66" s="13"/>
+      <c r="H66" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A67" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D67" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="B65" s="12"/>
-      <c r="D65" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E65" s="12"/>
-      <c r="H65" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="I65" s="12"/>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A66" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E66" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I66" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A67" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>53</v>
-      </c>
+      <c r="E67" s="19"/>
       <c r="H67" s="2" t="s">
-        <v>61</v>
+        <v>88</v>
       </c>
       <c r="I67" s="2" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="B68" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D70" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E70" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I70" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="H68" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="I68" s="2" t="s">
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A71" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B71" s="13"/>
+      <c r="D71" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E71" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I71" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A72" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D72" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E72" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E73" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D75" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E75" s="11"/>
+      <c r="H75" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A76" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="B76" s="13"/>
+      <c r="D76" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A77" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H77" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="I77" s="13"/>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A78" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D78" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E78" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I78" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A79" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I79" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D80" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E80" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I80" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="81" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D81" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E81" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I81" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="82" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D82" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E82" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I82" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="H69" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="I69" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A70" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B70" s="16"/>
-      <c r="D70" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E70" s="7"/>
-      <c r="H70" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="I70" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A71" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B71" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D71" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A72" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B72" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D72" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E72" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="H72" s="9" t="s">
+    <row r="83" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D83" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="E83" s="22" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="84" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D84" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="I72" s="10"/>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A73" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B73" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D73" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E73" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="H73" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I73" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D74" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E74" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H74" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="I74" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D75" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E75" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H75" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I75" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D76" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E76" s="7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D77" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E77" s="7" t="s">
-        <v>71</v>
+      <c r="E84" s="22" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="29">
+    <mergeCell ref="H77:I77"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D65:E65"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D19:E19"/>
+    <mergeCell ref="H56:I56"/>
+    <mergeCell ref="H65:I65"/>
     <mergeCell ref="H12:I12"/>
     <mergeCell ref="D30:F30"/>
     <mergeCell ref="A32:B32"/>
@@ -1779,13 +1970,14 @@
     <mergeCell ref="D43:E43"/>
     <mergeCell ref="H43:I43"/>
     <mergeCell ref="D54:F54"/>
+    <mergeCell ref="D56:E56"/>
     <mergeCell ref="A56:B56"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="H56:I56"/>
-    <mergeCell ref="H72:I72"/>
-    <mergeCell ref="A65:B65"/>
-    <mergeCell ref="A70:B70"/>
-    <mergeCell ref="H65:I65"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D75:E75"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
functional - assets CRUD(Manual)
</commit_message>
<xml_diff>
--- a/IMS_normalization.xlsx
+++ b/IMS_normalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\IMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7658D334-ADBF-4CBD-B2A2-4166B7C5FF41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9DC883-7F3D-4AF2-92DC-0909D3F2DC5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CDF4D7C-9BB1-444C-B0E6-E0178AB74584}"/>
   </bookViews>
@@ -464,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -490,21 +490,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -516,17 +504,26 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -864,11 +861,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -973,25 +970,25 @@
       <c r="J6" s="4"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="D12" s="18" t="s">
+      <c r="B12" s="14"/>
+      <c r="D12" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="19"/>
-      <c r="H12" s="14" t="s">
+      <c r="E12" s="17"/>
+      <c r="H12" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="I12" s="15"/>
+      <c r="I12" s="19"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
@@ -1102,10 +1099,10 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E19" s="15"/>
+      <c r="E19" s="19"/>
       <c r="H19" s="2" t="s">
         <v>88</v>
       </c>
@@ -1114,10 +1111,10 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="11"/>
+      <c r="B20" s="16"/>
       <c r="D20" s="3" t="s">
         <v>50</v>
       </c>
@@ -1162,10 +1159,10 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="11"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
@@ -1192,25 +1189,25 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D30" s="16" t="s">
+      <c r="D30" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="18" t="s">
+      <c r="A32" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="18"/>
-      <c r="D32" s="18" t="s">
+      <c r="B32" s="14"/>
+      <c r="D32" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="19"/>
-      <c r="H32" s="14" t="s">
+      <c r="E32" s="17"/>
+      <c r="H32" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="I32" s="15"/>
+      <c r="I32" s="19"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
@@ -1313,10 +1310,10 @@
       <c r="B38" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D38" s="14" t="s">
+      <c r="D38" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="15"/>
+      <c r="E38" s="19"/>
       <c r="H38" s="2" t="s">
         <v>88</v>
       </c>
@@ -1353,10 +1350,10 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="12" t="s">
+      <c r="A41" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="13"/>
+      <c r="B41" s="11"/>
       <c r="D41" s="2" t="s">
         <v>88</v>
       </c>
@@ -1379,10 +1376,10 @@
       <c r="B43" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D43" s="18" t="s">
+      <c r="D43" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="E43" s="19"/>
+      <c r="E43" s="17"/>
       <c r="H43" s="20"/>
       <c r="I43" s="21"/>
     </row>
@@ -1411,10 +1408,10 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="10" t="s">
+      <c r="A46" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B46" s="11"/>
+      <c r="B46" s="16"/>
       <c r="D46" s="8" t="s">
         <v>59</v>
       </c>
@@ -1473,25 +1470,25 @@
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D54" s="16" t="s">
+      <c r="D54" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="E54" s="17"/>
-      <c r="F54" s="17"/>
+      <c r="E54" s="13"/>
+      <c r="F54" s="13"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="12" t="s">
+      <c r="A56" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B56" s="13"/>
-      <c r="D56" s="18" t="s">
+      <c r="B56" s="11"/>
+      <c r="D56" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="E56" s="18"/>
-      <c r="H56" s="14" t="s">
+      <c r="E56" s="14"/>
+      <c r="H56" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="I56" s="15"/>
+      <c r="I56" s="19"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
@@ -1568,10 +1565,10 @@
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="10" t="s">
+      <c r="A61" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B61" s="11"/>
+      <c r="B61" s="16"/>
       <c r="D61" s="7" t="s">
         <v>88</v>
       </c>
@@ -1640,22 +1637,22 @@
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D65" s="22" t="s">
+      <c r="D65" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E65" s="22" t="s">
+      <c r="E65" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="H65" s="14" t="s">
+      <c r="H65" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="I65" s="15"/>
+      <c r="I65" s="19"/>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B66" s="13"/>
+      <c r="B66" s="11"/>
       <c r="H66" s="2" t="s">
         <v>59</v>
       </c>
@@ -1670,10 +1667,10 @@
       <c r="B67" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D67" s="18" t="s">
+      <c r="D67" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="E67" s="19"/>
+      <c r="E67" s="17"/>
       <c r="H67" s="2" t="s">
         <v>88</v>
       </c>
@@ -1736,10 +1733,10 @@
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A71" s="12" t="s">
+      <c r="A71" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B71" s="13"/>
+      <c r="B71" s="11"/>
       <c r="D71" s="7" t="s">
         <v>88</v>
       </c>
@@ -1808,10 +1805,10 @@
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D75" s="10" t="s">
+      <c r="D75" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="E75" s="11"/>
+      <c r="E75" s="16"/>
       <c r="H75" s="2" t="s">
         <v>88</v>
       </c>
@@ -1820,10 +1817,10 @@
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A76" s="12" t="s">
+      <c r="A76" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B76" s="13"/>
+      <c r="B76" s="11"/>
       <c r="D76" s="6" t="s">
         <v>31</v>
       </c>
@@ -1844,10 +1841,10 @@
       <c r="E77" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="H77" s="12" t="s">
+      <c r="H77" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I77" s="13"/>
+      <c r="I77" s="11"/>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
@@ -1932,23 +1929,36 @@
       </c>
     </row>
     <row r="83" spans="4:9" x14ac:dyDescent="0.3">
-      <c r="D83" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="E83" s="22" t="s">
+      <c r="D83" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E83" s="7" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="84" spans="4:9" x14ac:dyDescent="0.3">
-      <c r="D84" s="22" t="s">
+      <c r="D84" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="E84" s="22" t="s">
+      <c r="E84" s="7" t="s">
         <v>106</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D75:E75"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="D54:F54"/>
     <mergeCell ref="H77:I77"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D10:F10"/>
@@ -1965,19 +1975,6 @@
     <mergeCell ref="A41:B41"/>
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D75:E75"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Views for request and form - added
</commit_message>
<xml_diff>
--- a/IMS_normalization.xlsx
+++ b/IMS_normalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\IMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9DC883-7F3D-4AF2-92DC-0909D3F2DC5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F2A736-240A-42C5-A844-F6CE03AE4623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CDF4D7C-9BB1-444C-B0E6-E0178AB74584}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="111">
   <si>
     <t>ASSET</t>
   </si>
@@ -336,9 +336,6 @@
     <t>barcode_image_path_ID PK</t>
   </si>
   <si>
-    <t>barcode_image_path</t>
-  </si>
-  <si>
     <t>asset_status</t>
   </si>
   <si>
@@ -346,6 +343,21 @@
   </si>
   <si>
     <t>token_expiry</t>
+  </si>
+  <si>
+    <t>BOOELAN</t>
+  </si>
+  <si>
+    <t>asset_type_status</t>
+  </si>
+  <si>
+    <t>brand_status</t>
+  </si>
+  <si>
+    <t>role_status</t>
+  </si>
+  <si>
+    <t>unit_status</t>
   </si>
 </sst>
 </file>
@@ -495,22 +507,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -524,6 +530,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -861,11 +873,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -970,25 +982,25 @@
       <c r="J6" s="4"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="D12" s="14" t="s">
+      <c r="B12" s="12"/>
+      <c r="D12" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="17"/>
-      <c r="H12" s="18" t="s">
+      <c r="E12" s="13"/>
+      <c r="H12" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="I12" s="19"/>
+      <c r="I12" s="17"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
@@ -1099,10 +1111,10 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E19" s="19"/>
+      <c r="E19" s="17"/>
       <c r="H19" s="2" t="s">
         <v>88</v>
       </c>
@@ -1111,10 +1123,10 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="15"/>
       <c r="D20" s="3" t="s">
         <v>50</v>
       </c>
@@ -1189,25 +1201,25 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D30" s="12" t="s">
+      <c r="D30" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="14" t="s">
+      <c r="A32" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="14"/>
-      <c r="D32" s="14" t="s">
+      <c r="B32" s="12"/>
+      <c r="D32" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="17"/>
-      <c r="H32" s="18" t="s">
+      <c r="E32" s="13"/>
+      <c r="H32" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="I32" s="19"/>
+      <c r="I32" s="17"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
@@ -1310,10 +1322,10 @@
       <c r="B38" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D38" s="18" t="s">
+      <c r="D38" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="19"/>
+      <c r="E38" s="17"/>
       <c r="H38" s="2" t="s">
         <v>88</v>
       </c>
@@ -1376,12 +1388,12 @@
       <c r="B43" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D43" s="14" t="s">
+      <c r="D43" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="E43" s="17"/>
-      <c r="H43" s="20"/>
-      <c r="I43" s="21"/>
+      <c r="E43" s="13"/>
+      <c r="H43" s="18"/>
+      <c r="I43" s="19"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
@@ -1408,10 +1420,10 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="15" t="s">
+      <c r="A46" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B46" s="16"/>
+      <c r="B46" s="15"/>
       <c r="D46" s="8" t="s">
         <v>59</v>
       </c>
@@ -1470,25 +1482,25 @@
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D54" s="12" t="s">
+      <c r="D54" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="E54" s="13"/>
-      <c r="F54" s="13"/>
+      <c r="E54" s="21"/>
+      <c r="F54" s="21"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="10" t="s">
+      <c r="A56" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B56" s="11"/>
-      <c r="D56" s="14" t="s">
+      <c r="B56" s="16"/>
+      <c r="D56" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="E56" s="14"/>
-      <c r="H56" s="18" t="s">
+      <c r="E56" s="12"/>
+      <c r="H56" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="I56" s="19"/>
+      <c r="I56" s="17"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
@@ -1551,6 +1563,12 @@
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>107</v>
+      </c>
       <c r="D60" s="7" t="s">
         <v>59</v>
       </c>
@@ -1565,10 +1583,6 @@
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B61" s="16"/>
       <c r="D61" s="7" t="s">
         <v>88</v>
       </c>
@@ -1583,12 +1597,10 @@
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A62" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>39</v>
-      </c>
+      <c r="A62" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B62" s="15"/>
       <c r="D62" s="7" t="s">
         <v>88</v>
       </c>
@@ -1603,11 +1615,11 @@
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A63" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B63" s="7" t="s">
-        <v>41</v>
+      <c r="A63" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>39</v>
       </c>
       <c r="D63" s="7" t="s">
         <v>59</v>
@@ -1624,10 +1636,10 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D64" s="7" t="s">
         <v>59</v>
@@ -1637,22 +1649,30 @@
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A65" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="D65" s="7" t="s">
         <v>70</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="H65" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="H65" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="I65" s="19"/>
+      <c r="I65" s="17"/>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A66" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="B66" s="11"/>
+      <c r="A66" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="H66" s="2" t="s">
         <v>59</v>
       </c>
@@ -1661,16 +1681,10 @@
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A67" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D67" s="14" t="s">
+      <c r="D67" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="E67" s="17"/>
+      <c r="E67" s="13"/>
       <c r="H67" s="2" t="s">
         <v>88</v>
       </c>
@@ -1679,12 +1693,10 @@
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A68" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="A68" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B68" s="11"/>
       <c r="D68" s="6" t="s">
         <v>31</v>
       </c>
@@ -1699,11 +1711,11 @@
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A69" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>77</v>
+      <c r="A69" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>30</v>
       </c>
       <c r="D69" s="7" t="s">
         <v>59</v>
@@ -1719,6 +1731,12 @@
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="D70" s="7" t="s">
         <v>88</v>
       </c>
@@ -1733,10 +1751,12 @@
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A71" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B71" s="11"/>
+      <c r="A71" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>77</v>
+      </c>
       <c r="D71" s="7" t="s">
         <v>88</v>
       </c>
@@ -1751,11 +1771,11 @@
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A72" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>30</v>
+      <c r="A72" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>109</v>
       </c>
       <c r="D72" s="7" t="s">
         <v>88</v>
@@ -1771,12 +1791,6 @@
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A73" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="D73" s="7" t="s">
         <v>59</v>
       </c>
@@ -1791,12 +1805,10 @@
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A74" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>52</v>
-      </c>
+      <c r="A74" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B74" s="11"/>
       <c r="H74" s="2" t="s">
         <v>88</v>
       </c>
@@ -1805,10 +1817,16 @@
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D75" s="15" t="s">
+      <c r="A75" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D75" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="E75" s="16"/>
+      <c r="E75" s="15"/>
       <c r="H75" s="2" t="s">
         <v>88</v>
       </c>
@@ -1817,10 +1835,12 @@
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A76" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="B76" s="11"/>
+      <c r="A76" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="D76" s="6" t="s">
         <v>31</v>
       </c>
@@ -1829,11 +1849,11 @@
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A77" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>30</v>
+      <c r="A77" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="D77" s="7" t="s">
         <v>59</v>
@@ -1848,10 +1868,10 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D78" s="7" t="s">
         <v>59</v>
@@ -1867,12 +1887,6 @@
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A79" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="D79" s="7" t="s">
         <v>88</v>
       </c>
@@ -1887,6 +1901,10 @@
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A80" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B80" s="11"/>
       <c r="D80" s="7" t="s">
         <v>88</v>
       </c>
@@ -1900,7 +1918,13 @@
         <v>73</v>
       </c>
     </row>
-    <row r="81" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A81" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="D81" s="7" t="s">
         <v>59</v>
       </c>
@@ -1914,7 +1938,13 @@
         <v>74</v>
       </c>
     </row>
-    <row r="82" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A82" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>102</v>
+      </c>
       <c r="D82" s="7" t="s">
         <v>70</v>
       </c>
@@ -1928,37 +1958,25 @@
         <v>75</v>
       </c>
     </row>
-    <row r="83" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D83" s="7" t="s">
         <v>88</v>
       </c>
       <c r="E83" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="84" spans="4:9" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D84" s="7" t="s">
         <v>78</v>
       </c>
       <c r="E84" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D75:E75"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="A80:B80"/>
     <mergeCell ref="H77:I77"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D10:F10"/>
@@ -1975,6 +1993,18 @@
     <mergeCell ref="A41:B41"/>
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D75:E75"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A62:B62"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="A74:B74"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Print Barcode - Added
</commit_message>
<xml_diff>
--- a/IMS_normalization.xlsx
+++ b/IMS_normalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\IMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F2A736-240A-42C5-A844-F6CE03AE4623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB8DEC5-CACC-4053-BEDA-97C72568183E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CDF4D7C-9BB1-444C-B0E6-E0178AB74584}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="115">
   <si>
     <t>ASSET</t>
   </si>
@@ -237,9 +237,6 @@
     <t>status</t>
   </si>
   <si>
-    <t>BOOLEAN</t>
-  </si>
-  <si>
     <t>Session</t>
   </si>
   <si>
@@ -321,9 +318,6 @@
     <t>Purpose</t>
   </si>
   <si>
-    <t>request_note</t>
-  </si>
-  <si>
     <t>KLD_ID</t>
   </si>
   <si>
@@ -345,9 +339,6 @@
     <t>token_expiry</t>
   </si>
   <si>
-    <t>BOOELAN</t>
-  </si>
-  <si>
     <t>asset_type_status</t>
   </si>
   <si>
@@ -358,6 +349,27 @@
   </si>
   <si>
     <t>unit_status</t>
+  </si>
+  <si>
+    <t>brand_id FK</t>
+  </si>
+  <si>
+    <t>borrow_ID</t>
+  </si>
+  <si>
+    <t>ENUM</t>
+  </si>
+  <si>
+    <t>Borrowed</t>
+  </si>
+  <si>
+    <t>borrow_status</t>
+  </si>
+  <si>
+    <t>reponse_status</t>
+  </si>
+  <si>
+    <t>request_status</t>
   </si>
 </sst>
 </file>
@@ -476,7 +488,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -501,11 +513,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -522,6 +534,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -531,11 +549,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -851,21 +866,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DB240BC-D6BF-403C-8C3D-179145117FF2}">
-  <dimension ref="A2:J84"/>
+  <dimension ref="A2:J90"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.33203125" customWidth="1"/>
+    <col min="5" max="5" width="23.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" customWidth="1"/>
+    <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="22.109375" bestFit="1" customWidth="1"/>
@@ -873,11 +888,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -982,11 +997,11 @@
       <c r="J6" s="4"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
@@ -1000,7 +1015,7 @@
       <c r="H12" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="I12" s="17"/>
+      <c r="I12" s="19"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
@@ -1050,7 +1065,7 @@
         <v>36</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>46</v>
@@ -1064,7 +1079,7 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>33</v>
@@ -1084,13 +1099,13 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>34</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>56</v>
@@ -1104,7 +1119,7 @@
         <v>37</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>57</v>
@@ -1114,9 +1129,9 @@
       <c r="D19" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E19" s="17"/>
+      <c r="E19" s="19"/>
       <c r="H19" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>58</v>
@@ -1156,7 +1171,7 @@
         <v>41</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>52</v>
@@ -1164,17 +1179,17 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="11"/>
+      <c r="B25" s="18"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
@@ -1194,18 +1209,18 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D30" s="20" t="s">
+      <c r="D30" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="12" t="s">
@@ -1219,7 +1234,7 @@
       <c r="H32" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="I32" s="17"/>
+      <c r="I32" s="19"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
@@ -1269,7 +1284,7 @@
         <v>36</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>46</v>
@@ -1303,13 +1318,13 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B37" s="7" t="s">
         <v>33</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>56</v>
@@ -1317,7 +1332,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>34</v>
@@ -1325,9 +1340,9 @@
       <c r="D38" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="17"/>
+      <c r="E38" s="19"/>
       <c r="H38" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>57</v>
@@ -1347,7 +1362,7 @@
         <v>30</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>58</v>
@@ -1362,12 +1377,12 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="10" t="s">
+      <c r="A41" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="11"/>
+      <c r="B41" s="18"/>
       <c r="D41" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>52</v>
@@ -1392,12 +1407,12 @@
         <v>63</v>
       </c>
       <c r="E43" s="13"/>
-      <c r="H43" s="18"/>
-      <c r="I43" s="19"/>
+      <c r="H43" s="20"/>
+      <c r="I43" s="21"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>43</v>
@@ -1439,7 +1454,7 @@
         <v>39</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E47" s="8" t="s">
         <v>66</v>
@@ -1453,7 +1468,7 @@
         <v>41</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E48" s="8" t="s">
         <v>67</v>
@@ -1461,13 +1476,13 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B49" s="7" t="s">
         <v>40</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E49" s="8" t="s">
         <v>68</v>
@@ -1475,18 +1490,18 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D50" s="8" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D54" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="E54" s="21"/>
-      <c r="F54" s="21"/>
+      <c r="D54" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="E54" s="11"/>
+      <c r="F54" s="11"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" s="16" t="s">
@@ -1500,7 +1515,7 @@
       <c r="H56" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="I56" s="17"/>
+      <c r="I56" s="19"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
@@ -1539,12 +1554,12 @@
         <v>59</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>43</v>
@@ -1559,15 +1574,15 @@
         <v>59</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>107</v>
+      <c r="A60" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="D60" s="7" t="s">
         <v>59</v>
@@ -1584,13 +1599,13 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D61" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E61" s="7" t="s">
         <v>33</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I61" s="2" t="s">
         <v>56</v>
@@ -1602,13 +1617,13 @@
       </c>
       <c r="B62" s="15"/>
       <c r="D62" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E62" s="7" t="s">
         <v>34</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I62" s="2" t="s">
         <v>57</v>
@@ -1628,7 +1643,7 @@
         <v>62</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I63" s="2" t="s">
         <v>58</v>
@@ -1645,39 +1660,39 @@
         <v>59</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B65" s="7" t="s">
         <v>40</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H65" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="I65" s="17"/>
+        <v>88</v>
+      </c>
+      <c r="I65" s="19"/>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>59</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
@@ -1686,17 +1701,17 @@
       </c>
       <c r="E67" s="13"/>
       <c r="H67" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I67" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A68" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="B68" s="11"/>
+      <c r="A68" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="B68" s="18"/>
       <c r="D68" s="6" t="s">
         <v>31</v>
       </c>
@@ -1707,7 +1722,7 @@
         <v>60</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
@@ -1724,10 +1739,10 @@
         <v>47</v>
       </c>
       <c r="H69" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="I69" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="I69" s="2" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
@@ -1735,59 +1750,59 @@
         <v>59</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>59</v>
       </c>
       <c r="I70" s="2" t="s">
-        <v>45</v>
+        <v>108</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>59</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
@@ -1801,19 +1816,19 @@
         <v>59</v>
       </c>
       <c r="I73" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A74" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B74" s="18"/>
+      <c r="H74" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I74" s="2" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A74" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B74" s="11"/>
-      <c r="H74" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="I74" s="2" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
@@ -1828,10 +1843,10 @@
       </c>
       <c r="E75" s="15"/>
       <c r="H75" s="2" t="s">
-        <v>88</v>
+        <v>110</v>
       </c>
       <c r="I75" s="2" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
@@ -1847,10 +1862,16 @@
       <c r="E76" s="6" t="s">
         <v>30</v>
       </c>
+      <c r="H76" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="I76" s="22" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>52</v>
@@ -1861,52 +1882,46 @@
       <c r="E77" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="H77" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="I77" s="11"/>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E78" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="H78" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="B78" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D78" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E78" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="H78" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I78" s="3" t="s">
-        <v>30</v>
-      </c>
+      <c r="I78" s="18"/>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D79" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E79" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="H79" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="I79" s="2" t="s">
-        <v>72</v>
+      <c r="H79" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I79" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A80" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="B80" s="11"/>
+      <c r="A80" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B80" s="18"/>
       <c r="D80" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E80" s="7" t="s">
         <v>67</v>
@@ -1915,7 +1930,7 @@
         <v>59</v>
       </c>
       <c r="I80" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">
@@ -1929,13 +1944,13 @@
         <v>59</v>
       </c>
       <c r="E81" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="I81" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.3">
@@ -1943,41 +1958,86 @@
         <v>59</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D82" s="7" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="E82" s="7" t="s">
         <v>69</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I82" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D83" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E83" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
+      </c>
+      <c r="H83" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I83" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D84" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E84" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D86" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="E86" s="19"/>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D87" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D88" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D89" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D90" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
+    <mergeCell ref="D86:E86"/>
+    <mergeCell ref="H78:I78"/>
     <mergeCell ref="A80:B80"/>
-    <mergeCell ref="H77:I77"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="A12:B12"/>

</xml_diff>

<commit_message>
QR code - added
</commit_message>
<xml_diff>
--- a/IMS_normalization.xlsx
+++ b/IMS_normalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\IMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB8DEC5-CACC-4053-BEDA-97C72568183E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA193C5-6985-4F3E-875A-05513084F1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CDF4D7C-9BB1-444C-B0E6-E0178AB74584}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="134">
   <si>
     <t>ASSET</t>
   </si>
@@ -318,9 +318,6 @@
     <t>Purpose</t>
   </si>
   <si>
-    <t>KLD_ID</t>
-  </si>
-  <si>
     <t>barcode_image_path_ID FK</t>
   </si>
   <si>
@@ -370,6 +367,66 @@
   </si>
   <si>
     <t>request_status</t>
+  </si>
+  <si>
+    <t>borrow_date</t>
+  </si>
+  <si>
+    <t>borrow_time</t>
+  </si>
+  <si>
+    <t>due_date</t>
+  </si>
+  <si>
+    <t>due_time</t>
+  </si>
+  <si>
+    <t>message</t>
+  </si>
+  <si>
+    <t>message_ID PK</t>
+  </si>
+  <si>
+    <t>account_ID FK</t>
+  </si>
+  <si>
+    <t>TEXT</t>
+  </si>
+  <si>
+    <t>message_content</t>
+  </si>
+  <si>
+    <t>message_date</t>
+  </si>
+  <si>
+    <t>kld_email</t>
+  </si>
+  <si>
+    <t>borrower_name</t>
+  </si>
+  <si>
+    <t>date_added</t>
+  </si>
+  <si>
+    <t>subject</t>
+  </si>
+  <si>
+    <t>BOOLEAN</t>
+  </si>
+  <si>
+    <t>is_read</t>
+  </si>
+  <si>
+    <t>message_status</t>
+  </si>
+  <si>
+    <t>qr_image_path_ID FK</t>
+  </si>
+  <si>
+    <t>QR_code</t>
+  </si>
+  <si>
+    <t>qr_image_path_ID PK</t>
   </si>
 </sst>
 </file>
@@ -435,7 +492,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -484,11 +541,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -513,6 +579,18 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -522,26 +600,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -552,6 +618,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -866,7 +939,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DB240BC-D6BF-403C-8C3D-179145117FF2}">
-  <dimension ref="A2:J90"/>
+  <dimension ref="A2:J96"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -888,11 +961,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -997,25 +1070,25 @@
       <c r="J6" s="4"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="12"/>
-      <c r="D12" s="12" t="s">
+      <c r="B12" s="16"/>
+      <c r="D12" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="H12" s="16" t="s">
+      <c r="E12" s="19"/>
+      <c r="H12" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="I12" s="19"/>
+      <c r="I12" s="11"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
@@ -1126,10 +1199,10 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D19" s="16" t="s">
+      <c r="D19" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="E19" s="19"/>
+      <c r="E19" s="11"/>
       <c r="H19" s="2" t="s">
         <v>87</v>
       </c>
@@ -1138,10 +1211,10 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="15"/>
+      <c r="B20" s="18"/>
       <c r="D20" s="3" t="s">
         <v>50</v>
       </c>
@@ -1186,10 +1259,10 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="18"/>
+      <c r="B25" s="13"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
@@ -1216,25 +1289,25 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="12"/>
-      <c r="D32" s="12" t="s">
+      <c r="B32" s="16"/>
+      <c r="D32" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="13"/>
-      <c r="H32" s="16" t="s">
+      <c r="E32" s="19"/>
+      <c r="H32" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="I32" s="19"/>
+      <c r="I32" s="11"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
@@ -1337,10 +1410,10 @@
       <c r="B38" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D38" s="16" t="s">
+      <c r="D38" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="19"/>
+      <c r="E38" s="11"/>
       <c r="H38" s="2" t="s">
         <v>87</v>
       </c>
@@ -1377,10 +1450,10 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="17" t="s">
+      <c r="A41" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="18"/>
+      <c r="B41" s="13"/>
       <c r="D41" s="2" t="s">
         <v>87</v>
       </c>
@@ -1403,10 +1476,10 @@
       <c r="B43" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D43" s="12" t="s">
+      <c r="D43" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="E43" s="13"/>
+      <c r="E43" s="19"/>
       <c r="H43" s="20"/>
       <c r="I43" s="21"/>
     </row>
@@ -1435,10 +1508,10 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="14" t="s">
+      <c r="A46" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B46" s="15"/>
+      <c r="B46" s="18"/>
       <c r="D46" s="8" t="s">
         <v>59</v>
       </c>
@@ -1490,32 +1563,32 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D50" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D54" s="10" t="s">
+      <c r="D54" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="E54" s="11"/>
-      <c r="F54" s="11"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="16" t="s">
+      <c r="A56" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B56" s="16"/>
-      <c r="D56" s="12" t="s">
+      <c r="B56" s="10"/>
+      <c r="D56" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="E56" s="12"/>
-      <c r="H56" s="16" t="s">
+      <c r="E56" s="16"/>
+      <c r="H56" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="I56" s="19"/>
+      <c r="I56" s="11"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
@@ -1579,10 +1652,10 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D60" s="7" t="s">
         <v>59</v>
@@ -1612,10 +1685,10 @@
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A62" s="14" t="s">
+      <c r="A62" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B62" s="15"/>
+      <c r="B62" s="18"/>
       <c r="D62" s="7" t="s">
         <v>87</v>
       </c>
@@ -1660,7 +1733,7 @@
         <v>59</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
@@ -1670,23 +1743,29 @@
       <c r="B65" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D65" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="E65" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="H65" s="16" t="s">
+      <c r="D65" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="E65" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="H65" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="I65" s="19"/>
+      <c r="I65" s="11"/>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
+      </c>
+      <c r="D66" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="E66" s="23" t="s">
+        <v>126</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>59</v>
@@ -1696,33 +1775,29 @@
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D67" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="E67" s="13"/>
-      <c r="H67" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="I67" s="2" t="s">
-        <v>97</v>
+      <c r="D67" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E67" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="H67" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="I67" s="22" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A68" s="17" t="s">
+      <c r="A68" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B68" s="18"/>
-      <c r="D68" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E68" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="B68" s="13"/>
       <c r="H68" s="2" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>89</v>
+        <v>124</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
@@ -1732,17 +1807,15 @@
       <c r="B69" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D69" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E69" s="7" t="s">
-        <v>47</v>
-      </c>
+      <c r="D69" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E69" s="18"/>
       <c r="H69" s="2" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
@@ -1752,17 +1825,17 @@
       <c r="B70" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D70" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="E70" s="7" t="s">
-        <v>83</v>
+      <c r="D70" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="I70" s="2" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
@@ -1773,62 +1846,68 @@
         <v>76</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D72" s="7" t="s">
         <v>87</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D73" s="7" t="s">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>59</v>
       </c>
       <c r="I73" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A74" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B74" s="13"/>
+      <c r="D74" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E74" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I74" s="2" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A74" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="B74" s="18"/>
-      <c r="H74" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="I74" s="2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
@@ -1838,15 +1917,17 @@
       <c r="B75" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D75" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="E75" s="15"/>
+      <c r="D75" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E75" s="7" t="s">
+        <v>48</v>
+      </c>
       <c r="H75" s="2" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="I75" s="2" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
@@ -1856,17 +1937,11 @@
       <c r="B76" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D76" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E76" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H76" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="I76" s="22" t="s">
-        <v>114</v>
+      <c r="H76" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I76" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
@@ -1876,61 +1951,59 @@
       <c r="B77" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D77" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E77" s="7" t="s">
-        <v>65</v>
+      <c r="D77" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="E77" s="18"/>
+      <c r="H77" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D78" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E78" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="H78" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="I78" s="18"/>
+        <v>106</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D79" s="7" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="E79" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="H79" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H79" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="I79" s="13"/>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A80" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="B80" s="13"/>
+      <c r="D80" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E80" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="H80" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I79" s="3" t="s">
+      <c r="I80" s="3" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A80" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="B80" s="18"/>
-      <c r="D80" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="E80" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="H80" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="I80" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">
@@ -1941,16 +2014,16 @@
         <v>30</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="E81" s="7" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="H81" s="2" t="s">
         <v>59</v>
       </c>
       <c r="I81" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.3">
@@ -1958,85 +2031,221 @@
         <v>59</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D82" s="7" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E82" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="I82" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D83" s="7" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="E83" s="7" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="H83" s="2" t="s">
         <v>77</v>
       </c>
       <c r="I83" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A84" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="B84" s="24"/>
+      <c r="D84" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E84" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I84" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D84" s="7" t="s">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A85" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A86" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D86" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="E84" s="7" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D86" s="16" t="s">
+      <c r="E86" s="7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A87" s="25"/>
+      <c r="B87" s="25"/>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A88" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B88" s="11"/>
+      <c r="D88" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E88" s="13"/>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A89" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D89" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="E89" s="23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A90" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D90" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="E90" s="23" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A91" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D91" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="E91" s="23" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A92" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D92" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="E92" s="23" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A93" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D93" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="E93" s="23" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A94" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D94" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="E94" s="23" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A95" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D95" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="E95" s="23" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A96" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B96" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E86" s="19"/>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D87" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E87" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D88" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D89" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D90" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>112</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="D86:E86"/>
-    <mergeCell ref="H78:I78"/>
+  <mergeCells count="32">
+    <mergeCell ref="H79:I79"/>
+    <mergeCell ref="A84:B84"/>
+    <mergeCell ref="D77:E77"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A62:B62"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="A88:B88"/>
     <mergeCell ref="A80:B80"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D10:F10"/>
@@ -2051,20 +2260,6 @@
     <mergeCell ref="D30:F30"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D75:E75"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A62:B62"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="A74:B74"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>